<commit_message>
feat: enhance invoice handling with improved row selection and modal interactions
</commit_message>
<xml_diff>
--- a/gdt-aggregated-xlsx/hd_purchased_merged.xlsx
+++ b/gdt-aggregated-xlsx/hd_purchased_merged.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="502" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="502" uniqueCount="166">
   <si>
     <t>DANH SÁCH HÓA ĐƠN</t>
   </si>
@@ -115,7 +115,7 @@
     <t>Hóa đơn mới</t>
   </si>
   <si>
-    <t>Xăng E10 RON 95 Mức 3,36.265,Lít,22060,800000,KKKNT</t>
+    <t>Hàng hóa, dịch vụ - Xăng E10 RON 95 Mức 3 - 36.265 - Lít - 22.060 - 800.000 - KKKNT</t>
   </si>
   <si>
     <t>C26TBA</t>
@@ -136,7 +136,7 @@
     <t>53 Nguyễn Đức Thuận, Phường Tân Bình, Thành phố Hồ Chí Minh, Việt Nam</t>
   </si>
   <si>
-    <t>Dịch vụ sửa chữa,1,Gói,850000,850000,8%</t>
+    <t>Hàng hóa, dịch vụ - Dịch vụ sửa chữa - 1 - Gói - 850.000 - 850.000 - 8%</t>
   </si>
   <si>
     <t>3662</t>
@@ -145,7 +145,7 @@
     <t>05/06/2026</t>
   </si>
   <si>
-    <t>Dịch vụ phần mềm quản lý và lưu trữ dữ liệu theo học viên (01/06/2026 - 31/05/2027),1,Gói,1200000,1200000,KCT</t>
+    <t>Hàng hóa, dịch vụ - Dịch vụ phần mềm quản lý và lưu trữ dữ liệu theo học viên (01/06/2026 - 31/05/2027) - 1 - Gói - 1.200.000 - 1.200.000 - KCT</t>
   </si>
   <si>
     <t>3965</t>
@@ -154,7 +154,7 @@
     <t>17/06/2026</t>
   </si>
   <si>
-    <t>Dịch vụ phần mềm quản lý và lưu trữ dữ liệu theo học viên (15/06/2026 - 14/06/2027),3,Gói,1200000,3600000,KCT</t>
+    <t>Hàng hóa, dịch vụ - Dịch vụ phần mềm quản lý và lưu trữ dữ liệu theo học viên (15/06/2026 - 14/06/2027) - 3 - Gói - 1.200.000 - 3.600.000 - KCT</t>
   </si>
   <si>
     <t>4221</t>
@@ -163,17 +163,13 @@
     <t>26/06/2026</t>
   </si>
   <si>
-    <t xml:space="preserve">Dịch vụ phần mềm quản lý và lưu trữ dữ liệu theo học viên (01/07/2026 - 30/06/2027),14,Gói,1200000,16800000,KCT
-Dịch vụ phần mềm quản lý và lưu trữ dữ liệu theo học viên (15/07/2026 - 14/07/2027),17,Gói,1200000,20400000,KCT</t>
+    <t xml:space="preserve">Hàng hóa, dịch vụ - Dịch vụ phần mềm quản lý và lưu trữ dữ liệu theo học viên (01/07/2026 - 30/06/2027) - 14 - Gói - 1.200.000 - 16.800.000 - KCT
+Hàng hóa, dịch vụ - Dịch vụ phần mềm quản lý và lưu trữ dữ liệu theo học viên (15/07/2026 - 14/07/2027) - 17 - Gói - 1.200.000 - 20.400.000 - KCT</t>
   </si>
   <si>
     <t>4252</t>
   </si>
   <si>
-    <t xml:space="preserve">Dịch vụ phần mềm quản lý và lưu trữ dữ liệu theo học viên (01/07/2026 - 30/06/2027),,,,,
-Dịch vụ phần mềm quản lý và lưu trữ dữ liệu theo học viên (15/07/2026 - 14/07/2027),,,,,</t>
-  </si>
-  <si>
     <t>C26TBD</t>
   </si>
   <si>
@@ -192,9 +188,6 @@
     <t>53 Nguyễn Đức Thuận, Phường Tân Bình,  TP Hồ Chí Minh, Việt Nam</t>
   </si>
   <si>
-    <t>Dịch vụ sửa chữa,,,,,</t>
-  </si>
-  <si>
     <t>114100</t>
   </si>
   <si>
@@ -207,33 +200,30 @@
     <t>04/06/2026</t>
   </si>
   <si>
-    <t xml:space="preserve">DO.TTKD037_KD05/M03/2600660900 - Bảo hiểm bắt buộc TNDS của chủ xe 51C45909,,,,,
-DO.TTKD037_KD05/M03/2600660900 - Bảo hiểm Tai nạn lái xe và người ngồi trên xe,,,,,</t>
+    <t xml:space="preserve">Hàng hóa, dịch vụ - DO.TTKD037_KD05/M03/2600660900 - Bảo hiểm bắt buộc TNDS của chủ xe 51C45909 - 1 - đơn vị - 4.800.000 - 4.800.000 - 10%
+Hàng hóa, dịch vụ - DO.TTKD037_KD05/M03/2600660900 - Bảo hiểm Tai nạn lái xe và người ngồi trên xe - 1 - đơn vị - 20.000 - 20.000 - KCT</t>
   </si>
   <si>
     <t>120251</t>
   </si>
   <si>
-    <t>Dịch vụ phần mềm quản lý và lưu trữ dữ liệu theo học viên (01/06/2026 - 31/05/2027),,,,,</t>
-  </si>
-  <si>
     <t>123722</t>
   </si>
   <si>
     <t>07/06/2026</t>
   </si>
   <si>
-    <t xml:space="preserve">Sửa chữa xe BKS 51A91775,,,,,
-Bảo dưỡng cấp trung bình kdd,,,,,
-Dầu máy SP 10W-30 (phuy 208L),,,,,
-Gioăng làm kín ốc xả dầu,,,,,
-Lọc dầu động cơ,,,,,</t>
+    <t xml:space="preserve">Ghi chú, diễn giải - Sửa chữa xe BKS 51A91775 - 0 - 0%
+Hàng hóa, dịch vụ - Bảo dưỡng cấp trung bình kdd - 1 - Lượt - 250.000 - 250.000 - 8%
+Hàng hóa, dịch vụ - Dầu máy SP 10W-30 (phuy 208L) - 3.7 - Lít - 104.400 - 386.280 - 8%
+Hàng hóa, dịch vụ - Gioăng làm kín ốc xả dầu - 1 - Cái - 10.800 - 10.800 - 8%
+Hàng hóa, dịch vụ - Lọc dầu động cơ - 1 - Cái - 187.200 - 187.200 - 8%</t>
   </si>
   <si>
     <t>123723</t>
   </si>
   <si>
-    <t>Xăng E10 RON95 Mức 3,35.244,Lít,22330,787000,KKKNT</t>
+    <t>Hàng hóa, dịch vụ - Xăng E10 RON95 Mức 3 - 35.244 - Lít - 22.330 - 787.000 - KKKNT</t>
   </si>
   <si>
     <t>127104</t>
@@ -248,13 +238,13 @@
     <t>14/06/2026</t>
   </si>
   <si>
-    <t>Kiểm định Ô tô từ 9 chỗ trở xuống: 51K-126.36,,,,,</t>
+    <t>Hàng hóa, dịch vụ - Kiểm định Ô tô từ 9 chỗ trở xuống: 51K-126.36 - 1 - Lượt - 227.273 - 227.273 - 8%</t>
   </si>
   <si>
     <t>134472</t>
   </si>
   <si>
-    <t>Xăng E10 RON95 Mức 3,22.665,Lít,22060,500000,KKKNT</t>
+    <t>Hàng hóa, dịch vụ - Xăng E10 RON95 Mức 3 - 22.665 - Lít - 22.060 - 500.000 - KKKNT</t>
   </si>
   <si>
     <t>136322</t>
@@ -266,22 +256,19 @@
     <t>139907</t>
   </si>
   <si>
-    <t>Dịch vụ phần mềm quản lý và lưu trữ dữ liệu theo học viên (15/06/2026 - 14/06/2027),,,,,</t>
-  </si>
-  <si>
     <t>145668</t>
   </si>
   <si>
     <t>21/06/2026</t>
   </si>
   <si>
-    <t xml:space="preserve">Sửa chữa xe BKS 51H77732,,,,,
-Bảo dưỡng cấp trung bình ( chỉ vệ sinh thắng đĩa),,,,,
-Dung dịch tẩy rửa bố thắng,,,,,
-Dầu máy SP 10W-30 (phuy 208L),,,,,
-Lọc dầu động cơ,,,,,
-Gioăng làm kín ốc xả dầu,,,,,
-Lõi lọc gió động cơ,,,,,</t>
+    <t xml:space="preserve">Ghi chú, diễn giải - Sửa chữa xe BKS 51H77732 - 0 - 0%
+Hàng hóa, dịch vụ - Bảo dưỡng cấp trung bình ( chỉ vệ sinh thắng đĩa) - 1 - Lượt - 380.000 - 380.000 - 8%
+Hàng hóa, dịch vụ - Dung dịch tẩy rửa bố thắng - 1 - Chai - 90.900 - 90.900 - 8%
+Hàng hóa, dịch vụ - Dầu máy SP 10W-30 (phuy 208L) - 3.3 - Lít - 104.400 - 344.520 - 8%
+Hàng hóa, dịch vụ - Lọc dầu động cơ - 1 - Cái - 187.200 - 187.200 - 8%
+Hàng hóa, dịch vụ - Gioăng làm kín ốc xả dầu - 1 - Cái - 10.800 - 10.800 - 8%
+Hàng hóa, dịch vụ - Lõi lọc gió động cơ - 1 - Cái - 369.900 - 369.900 - 8%</t>
   </si>
   <si>
     <t>147715</t>
@@ -290,7 +277,7 @@
     <t>23/06/2026</t>
   </si>
   <si>
-    <t>Xăng E10 RON95 Mức 3,26.409,Lít,20750,548000,KKKNT</t>
+    <t>Hàng hóa, dịch vụ - Xăng E10 RON95 Mức 3 - 26.409 - Lít - 20.750 - 548.000 - KKKNT</t>
   </si>
   <si>
     <t>149230</t>
@@ -299,7 +286,7 @@
     <t>24/06/2026</t>
   </si>
   <si>
-    <t>Xăng E10 RON95 Mức 3,19.277,Lít,20750,400000,KKKNT</t>
+    <t>Hàng hóa, dịch vụ - Xăng E10 RON95 Mức 3 - 19.277 - Lít - 20.750 - 400.000 - KKKNT</t>
   </si>
   <si>
     <t>159219</t>
@@ -308,7 +295,7 @@
     <t>30/06/2026</t>
   </si>
   <si>
-    <t>Xăng E10 RON95 Mức 3,25.113,Lít,19910,500000,KKKNT</t>
+    <t>Hàng hóa, dịch vụ - Xăng E10 RON95 Mức 3 - 25.113 - Lít - 19.910 - 500.000 - KKKNT</t>
   </si>
   <si>
     <t>C26TTC</t>
@@ -326,10 +313,6 @@
     <t>Trung tâm giáo dục nghề nghiệp Bách Việt</t>
   </si>
   <si>
-    <t xml:space="preserve">DO.TTKD037_KD05/M03/2600660900 - Bảo hiểm bắt buộc TNDS của chủ xe 51C45909,1,đơn vị,4800000,4800000,10%
-DO.TTKD037_KD05/M03/2600660900 - Bảo hiểm Tai nạn lái xe và người ngồi trên xe,1,đơn vị,20000,20000,KCT</t>
-  </si>
-  <si>
     <t>C26TSS</t>
   </si>
   <si>
@@ -363,9 +346,6 @@
     <t>53 Nguyễn Đức Thuận, phường Tân Bình, Tp. Hồ Chí Minh</t>
   </si>
   <si>
-    <t>Xăng E10 RON95 Mức 3,,,,,</t>
-  </si>
-  <si>
     <t>2</t>
   </si>
   <si>
@@ -384,13 +364,13 @@
     <t>53 Nguyễn Đức Thuận, Phường Tân Bình, TP Hồ Chí Minh</t>
   </si>
   <si>
-    <t/>
+    <t>Hàng hóa, dịch vụ - Thu tiền ôn tập trên sân và xe có thiết bị. “Đã giảm 52.200 đồng tương ứng 20% mức tỷ lệ % để tính thuế giá trị gia tăng theo nghị quyết số 204/2025/QH15”. - 9 - Giờ - 580.000 - 5.220.000</t>
   </si>
   <si>
     <t>7948</t>
   </si>
   <si>
-    <t>Thu tiền ôn tập trên sân và xe có thiết bị. “Đã giảm 49.300 đồng tương ứng 20% mức tỷ lệ % để tính thuế giá trị gia tăng theo nghị quyết số 204/2025/QH15”.,8.5,Giờ,580000,4930000,</t>
+    <t>Hàng hóa, dịch vụ - Thu tiền ôn tập trên sân và xe có thiết bị. “Đã giảm 49.300 đồng tương ứng 20% mức tỷ lệ % để tính thuế giá trị gia tăng theo nghị quyết số 204/2025/QH15”. - 8.5 - Giờ - 580.000 - 4.930.000</t>
   </si>
   <si>
     <t>C26TSH</t>
@@ -426,11 +406,11 @@
     <t>Trung Tâm Giáo Dục Nghề Nghiệp Bách Việt</t>
   </si>
   <si>
-    <t xml:space="preserve">Sửa chữa xe BKS 51A91775,,,,0,0%
-Bảo dưỡng cấp trung bình  kdd,1,Lượt,250000,250000,8%
-Dầu máy SP 10W-30 (phuy 208L),3.7,Lít,104400,386280,8%
-Gioăng làm kín ốc xả dầu,1,Cái,10800,10800,8%
-Lọc dầu động cơ,1,Cái,187200,187200,8%</t>
+    <t xml:space="preserve">Ghi chú, diễn giải - Sửa chữa xe BKS 51A91775 - 0 - 0%
+Hàng hóa, dịch vụ - Bảo dưỡng cấp trung bình  kdd - 1 - Lượt - 250.000 - 250.000 - 8%
+Hàng hóa, dịch vụ - Dầu máy SP 10W-30 (phuy 208L) - 3.7 - Lít - 104.400 - 386.280 - 8%
+Hàng hóa, dịch vụ - Gioăng làm kín ốc xả dầu - 1 - Cái - 10.800 - 10.800 - 8%
+Hàng hóa, dịch vụ - Lọc dầu động cơ - 1 - Cái - 187.200 - 187.200 - 8%</t>
   </si>
   <si>
     <t>9203</t>
@@ -445,13 +425,13 @@
     <t>53 Nguyễn Đức Thuận, Phường Tân Bình, Thành Phố  Hồ Chí Minh, Việt Nam</t>
   </si>
   <si>
-    <t xml:space="preserve">Sửa chữa xe BKS 51H77732,,,,0,0%
-Bảo dưỡng cấp trung bình  ( chỉ vệ sinh thắng đĩa),1,Lượt,380000,380000,8%
-Dung dịch tẩy rửa bố thắng,1,Chai,90900,90900,8%
-Dầu máy SP 10W-30 (phuy 208L),3.3,Lít,104400,344520,8%
-Lọc dầu động cơ,1,Cái,187200,187200,8%
-Gioăng làm kín ốc xả dầu,1,Cái,10800,10800,8%
-Lõi lọc gió động cơ,1,Cái,369900,369900,8%</t>
+    <t xml:space="preserve">Ghi chú, diễn giải - Sửa chữa xe BKS 51H77732 - 0 - 0%
+Hàng hóa, dịch vụ - Bảo dưỡng cấp trung bình  ( chỉ vệ sinh thắng đĩa) - 1 - Lượt - 380.000 - 380.000 - 8%
+Hàng hóa, dịch vụ - Dung dịch tẩy rửa bố thắng - 1 - Chai - 90.900 - 90.900 - 8%
+Hàng hóa, dịch vụ - Dầu máy SP 10W-30 (phuy 208L) - 3.3 - Lít - 104.400 - 344.520 - 8%
+Hàng hóa, dịch vụ - Lọc dầu động cơ - 1 - Cái - 187.200 - 187.200 - 8%
+Hàng hóa, dịch vụ - Gioăng làm kín ốc xả dầu - 1 - Cái - 10.800 - 10.800 - 8%
+Hàng hóa, dịch vụ - Lõi lọc gió động cơ - 1 - Cái - 369.900 - 369.900 - 8%</t>
   </si>
   <si>
     <t>C26TYY</t>
@@ -499,7 +479,7 @@
     <t>53 Nguyễn Đức Thuận, Phường Tân Bình, Thành phố  Hồ Chí Minh, Việt Nam</t>
   </si>
   <si>
-    <t>Ắc quy GS MF 85D26L,1,Cái,1666667,1666667,8%</t>
+    <t>Hàng hóa, dịch vụ - Ắc quy GS MF 85D26L - 1 - Cái - 1.666.667 - 1.666.667 - 8%</t>
   </si>
   <si>
     <t>C26THL</t>
@@ -554,9 +534,6 @@
   </si>
   <si>
     <t>53 Nguyễn Đức Thuận, Phường Tân Bình, Thành Phố Hồ Chí Minh, Việt Nam</t>
-  </si>
-  <si>
-    <t>Kiểm định Ô tô từ 9 chỗ trở xuống: 51K-126.36,1,Lượt,227273,227273,8%</t>
   </si>
 </sst>
 </file>
@@ -1110,7 +1087,7 @@
         <v>32</v>
       </c>
       <c r="S12" s="4" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="13" spans="1:19" x14ac:dyDescent="0.25">
@@ -1121,19 +1098,19 @@
         <v>21</v>
       </c>
       <c r="C13" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="D13" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="E13" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="E13" s="3" t="s">
+      <c r="F13" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="F13" s="3" t="s">
+      <c r="G13" s="4" t="s">
         <v>55</v>
-      </c>
-      <c r="G13" s="4" t="s">
-        <v>56</v>
       </c>
       <c r="H13" s="3" t="s">
         <v>27</v>
@@ -1142,7 +1119,7 @@
         <v>28</v>
       </c>
       <c r="J13" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="K13" s="5">
         <v>530000</v>
@@ -1167,7 +1144,7 @@
         <v>32</v>
       </c>
       <c r="S13" s="4" t="s">
-        <v>58</v>
+        <v>40</v>
       </c>
     </row>
     <row r="14" spans="1:19" x14ac:dyDescent="0.25">
@@ -1178,19 +1155,19 @@
         <v>21</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="F14" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="G14" s="4" t="s">
         <v>55</v>
-      </c>
-      <c r="G14" s="4" t="s">
-        <v>56</v>
       </c>
       <c r="H14" s="3" t="s">
         <v>27</v>
@@ -1199,7 +1176,7 @@
         <v>28</v>
       </c>
       <c r="J14" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="K14" s="5">
         <v>660019</v>
@@ -1224,7 +1201,7 @@
         <v>32</v>
       </c>
       <c r="S14" s="4" t="s">
-        <v>58</v>
+        <v>40</v>
       </c>
     </row>
     <row r="15" spans="1:19" x14ac:dyDescent="0.25">
@@ -1235,19 +1212,19 @@
         <v>21</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="F15" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="G15" s="4" t="s">
         <v>55</v>
-      </c>
-      <c r="G15" s="4" t="s">
-        <v>56</v>
       </c>
       <c r="H15" s="3" t="s">
         <v>27</v>
@@ -1256,7 +1233,7 @@
         <v>28</v>
       </c>
       <c r="J15" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="K15" s="5">
         <v>420000</v>
@@ -1281,7 +1258,7 @@
         <v>32</v>
       </c>
       <c r="S15" s="4" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.25">
@@ -1292,19 +1269,19 @@
         <v>21</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="E16" s="3" t="s">
         <v>42</v>
       </c>
       <c r="F16" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="G16" s="4" t="s">
         <v>55</v>
-      </c>
-      <c r="G16" s="4" t="s">
-        <v>56</v>
       </c>
       <c r="H16" s="3" t="s">
         <v>27</v>
@@ -1313,7 +1290,7 @@
         <v>28</v>
       </c>
       <c r="J16" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="K16" s="5">
         <v>700023</v>
@@ -1338,7 +1315,7 @@
         <v>32</v>
       </c>
       <c r="S16" s="4" t="s">
-        <v>65</v>
+        <v>43</v>
       </c>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.25">
@@ -1349,19 +1326,19 @@
         <v>21</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="F17" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="G17" s="4" t="s">
         <v>55</v>
-      </c>
-      <c r="G17" s="4" t="s">
-        <v>56</v>
       </c>
       <c r="H17" s="3" t="s">
         <v>27</v>
@@ -1370,7 +1347,7 @@
         <v>28</v>
       </c>
       <c r="J17" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="K17" s="5">
         <v>350000</v>
@@ -1395,7 +1372,7 @@
         <v>32</v>
       </c>
       <c r="S17" s="4" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
     </row>
     <row r="18" spans="1:19" x14ac:dyDescent="0.25">
@@ -1406,19 +1383,19 @@
         <v>21</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="F18" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="G18" s="4" t="s">
         <v>55</v>
-      </c>
-      <c r="G18" s="4" t="s">
-        <v>56</v>
       </c>
       <c r="H18" s="3" t="s">
         <v>27</v>
@@ -1427,7 +1404,7 @@
         <v>28</v>
       </c>
       <c r="J18" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="K18" s="5">
         <v>787000</v>
@@ -1452,7 +1429,7 @@
         <v>32</v>
       </c>
       <c r="S18" s="4" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.25">
@@ -1463,19 +1440,19 @@
         <v>21</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="F19" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="G19" s="4" t="s">
         <v>55</v>
-      </c>
-      <c r="G19" s="4" t="s">
-        <v>56</v>
       </c>
       <c r="H19" s="3" t="s">
         <v>27</v>
@@ -1484,7 +1461,7 @@
         <v>28</v>
       </c>
       <c r="J19" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="K19" s="5">
         <v>699956</v>
@@ -1509,7 +1486,7 @@
         <v>32</v>
       </c>
       <c r="S19" s="4" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
     </row>
     <row r="20" spans="1:19" x14ac:dyDescent="0.25">
@@ -1520,19 +1497,19 @@
         <v>21</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="F20" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="G20" s="4" t="s">
         <v>55</v>
-      </c>
-      <c r="G20" s="4" t="s">
-        <v>56</v>
       </c>
       <c r="H20" s="3" t="s">
         <v>27</v>
@@ -1541,7 +1518,7 @@
         <v>28</v>
       </c>
       <c r="J20" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="K20" s="5">
         <v>535000</v>
@@ -1566,7 +1543,7 @@
         <v>32</v>
       </c>
       <c r="S20" s="4" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
     </row>
     <row r="21" spans="1:19" x14ac:dyDescent="0.25">
@@ -1577,19 +1554,19 @@
         <v>21</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="F21" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="G21" s="4" t="s">
         <v>55</v>
-      </c>
-      <c r="G21" s="4" t="s">
-        <v>56</v>
       </c>
       <c r="H21" s="3" t="s">
         <v>27</v>
@@ -1598,7 +1575,7 @@
         <v>28</v>
       </c>
       <c r="J21" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="K21" s="5">
         <v>500000</v>
@@ -1623,7 +1600,7 @@
         <v>32</v>
       </c>
       <c r="S21" s="4" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="22" spans="1:19" x14ac:dyDescent="0.25">
@@ -1634,19 +1611,19 @@
         <v>21</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="F22" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="G22" s="4" t="s">
         <v>55</v>
-      </c>
-      <c r="G22" s="4" t="s">
-        <v>56</v>
       </c>
       <c r="H22" s="3" t="s">
         <v>27</v>
@@ -1655,7 +1632,7 @@
         <v>28</v>
       </c>
       <c r="J22" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="K22" s="5">
         <v>514373</v>
@@ -1680,7 +1657,7 @@
         <v>32</v>
       </c>
       <c r="S22" s="4" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
     </row>
     <row r="23" spans="1:19" x14ac:dyDescent="0.25">
@@ -1691,19 +1668,19 @@
         <v>21</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="E23" s="3" t="s">
         <v>45</v>
       </c>
       <c r="F23" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="G23" s="4" t="s">
         <v>55</v>
-      </c>
-      <c r="G23" s="4" t="s">
-        <v>56</v>
       </c>
       <c r="H23" s="3" t="s">
         <v>27</v>
@@ -1712,7 +1689,7 @@
         <v>28</v>
       </c>
       <c r="J23" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="K23" s="5">
         <v>700000</v>
@@ -1737,7 +1714,7 @@
         <v>32</v>
       </c>
       <c r="S23" s="4" t="s">
-        <v>81</v>
+        <v>46</v>
       </c>
     </row>
     <row r="24" spans="1:19" x14ac:dyDescent="0.25">
@@ -1748,19 +1725,19 @@
         <v>21</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="F24" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="G24" s="4" t="s">
         <v>55</v>
-      </c>
-      <c r="G24" s="4" t="s">
-        <v>56</v>
       </c>
       <c r="H24" s="3" t="s">
         <v>27</v>
@@ -1769,7 +1746,7 @@
         <v>28</v>
       </c>
       <c r="J24" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="K24" s="5">
         <v>584008</v>
@@ -1794,7 +1771,7 @@
         <v>32</v>
       </c>
       <c r="S24" s="4" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
     </row>
     <row r="25" spans="1:19" x14ac:dyDescent="0.25">
@@ -1805,19 +1782,19 @@
         <v>21</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="F25" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="G25" s="4" t="s">
         <v>55</v>
-      </c>
-      <c r="G25" s="4" t="s">
-        <v>56</v>
       </c>
       <c r="H25" s="3" t="s">
         <v>27</v>
@@ -1826,7 +1803,7 @@
         <v>28</v>
       </c>
       <c r="J25" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="K25" s="5">
         <v>548000</v>
@@ -1851,7 +1828,7 @@
         <v>32</v>
       </c>
       <c r="S25" s="4" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.25">
@@ -1862,19 +1839,19 @@
         <v>21</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="F26" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="G26" s="4" t="s">
         <v>55</v>
-      </c>
-      <c r="G26" s="4" t="s">
-        <v>56</v>
       </c>
       <c r="H26" s="3" t="s">
         <v>27</v>
@@ -1883,7 +1860,7 @@
         <v>28</v>
       </c>
       <c r="J26" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="K26" s="5">
         <v>400000</v>
@@ -1908,7 +1885,7 @@
         <v>32</v>
       </c>
       <c r="S26" s="4" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
     </row>
     <row r="27" spans="1:19" x14ac:dyDescent="0.25">
@@ -1919,19 +1896,19 @@
         <v>21</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="F27" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="G27" s="4" t="s">
         <v>55</v>
-      </c>
-      <c r="G27" s="4" t="s">
-        <v>56</v>
       </c>
       <c r="H27" s="3" t="s">
         <v>27</v>
@@ -1940,7 +1917,7 @@
         <v>28</v>
       </c>
       <c r="J27" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="K27" s="5">
         <v>500000</v>
@@ -1965,7 +1942,7 @@
         <v>32</v>
       </c>
       <c r="S27" s="4" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
     </row>
     <row r="28" spans="1:19" x14ac:dyDescent="0.25">
@@ -1976,25 +1953,25 @@
         <v>21</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="E28" s="3" t="s">
         <v>42</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="G28" s="4" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="H28" s="3" t="s">
         <v>27</v>
       </c>
       <c r="I28" s="4" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="J28" s="4" t="s">
         <v>29</v>
@@ -2022,7 +1999,7 @@
         <v>32</v>
       </c>
       <c r="S28" s="4" t="s">
-        <v>99</v>
+        <v>61</v>
       </c>
     </row>
     <row r="29" spans="1:19" x14ac:dyDescent="0.25">
@@ -2033,25 +2010,25 @@
         <v>21</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="G29" s="4" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="H29" s="3" t="s">
         <v>27</v>
       </c>
       <c r="I29" s="4" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="J29" s="4" t="s">
         <v>29</v>
@@ -2079,7 +2056,7 @@
         <v>32</v>
       </c>
       <c r="S29" s="4" t="s">
-        <v>81</v>
+        <v>46</v>
       </c>
     </row>
     <row r="30" spans="1:19" x14ac:dyDescent="0.25">
@@ -2090,28 +2067,28 @@
         <v>21</v>
       </c>
       <c r="C30" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="E30" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="F30" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="G30" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="H30" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="I30" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="J30" s="4" t="s">
         <v>105</v>
-      </c>
-      <c r="D30" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="E30" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="F30" s="3" t="s">
-        <v>108</v>
-      </c>
-      <c r="G30" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="H30" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="I30" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="J30" s="4" t="s">
-        <v>110</v>
       </c>
       <c r="K30" s="5">
         <v>1354545</v>
@@ -2134,7 +2111,7 @@
         <v>32</v>
       </c>
       <c r="S30" s="4" t="s">
-        <v>111</v>
+        <v>74</v>
       </c>
     </row>
     <row r="31" spans="1:19" x14ac:dyDescent="0.25">
@@ -2142,31 +2119,31 @@
         <v>25</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="F31" s="3" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="G31" s="4" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="H31" s="3" t="s">
         <v>27</v>
       </c>
       <c r="I31" s="4" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="J31" s="4" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="K31" s="5"/>
       <c r="L31" s="5"/>
@@ -2187,7 +2164,7 @@
         <v>32</v>
       </c>
       <c r="S31" s="4" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
     </row>
     <row r="32" spans="1:19" x14ac:dyDescent="0.25">
@@ -2195,31 +2172,31 @@
         <v>26</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="C32" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="D32" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="D32" s="3" t="s">
-        <v>119</v>
-      </c>
       <c r="E32" s="3" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="F32" s="3" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="G32" s="4" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="H32" s="3" t="s">
         <v>27</v>
       </c>
       <c r="I32" s="4" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="J32" s="4" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="K32" s="5"/>
       <c r="L32" s="5"/>
@@ -2240,7 +2217,7 @@
         <v>32</v>
       </c>
       <c r="S32" s="4" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
     </row>
     <row r="33" spans="1:19" x14ac:dyDescent="0.25">
@@ -2251,19 +2228,19 @@
         <v>21</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="F33" s="3" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="G33" s="4" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="H33" s="3" t="s">
         <v>27</v>
@@ -2272,7 +2249,7 @@
         <v>28</v>
       </c>
       <c r="J33" s="4" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="K33" s="5">
         <v>138481482</v>
@@ -2297,7 +2274,7 @@
         <v>32</v>
       </c>
       <c r="S33" s="4" t="s">
-        <v>81</v>
+        <v>46</v>
       </c>
     </row>
     <row r="34" spans="1:19" x14ac:dyDescent="0.25">
@@ -2308,25 +2285,25 @@
         <v>21</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="G34" s="4" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="H34" s="3" t="s">
         <v>27</v>
       </c>
       <c r="I34" s="4" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="J34" s="4" t="s">
         <v>29</v>
@@ -2352,7 +2329,7 @@
         <v>32</v>
       </c>
       <c r="S34" s="4" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
     </row>
     <row r="35" spans="1:19" x14ac:dyDescent="0.25">
@@ -2363,25 +2340,25 @@
         <v>21</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="G35" s="4" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="H35" s="3" t="s">
         <v>27</v>
       </c>
       <c r="I35" s="4" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="J35" s="4" t="s">
         <v>29</v>
@@ -2407,7 +2384,7 @@
         <v>32</v>
       </c>
       <c r="S35" s="4" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
     </row>
     <row r="36" spans="1:19" x14ac:dyDescent="0.25">
@@ -2418,19 +2395,19 @@
         <v>21</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="G36" s="4" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="H36" s="3" t="s">
         <v>27</v>
@@ -2439,7 +2416,7 @@
         <v>28</v>
       </c>
       <c r="J36" s="4" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="K36" s="5">
         <v>1383320</v>
@@ -2462,7 +2439,7 @@
         <v>32</v>
       </c>
       <c r="S36" s="4" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
     </row>
     <row r="37" spans="1:19" x14ac:dyDescent="0.25">
@@ -2473,25 +2450,25 @@
         <v>21</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="G37" s="4" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="H37" s="3" t="s">
         <v>27</v>
       </c>
       <c r="I37" s="4" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="J37" s="4" t="s">
         <v>39</v>
@@ -2519,7 +2496,7 @@
         <v>32</v>
       </c>
       <c r="S37" s="4" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
     </row>
     <row r="38" spans="1:19" x14ac:dyDescent="0.25">
@@ -2530,19 +2507,19 @@
         <v>21</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="G38" s="4" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="H38" s="3" t="s">
         <v>27</v>
@@ -2576,7 +2553,7 @@
         <v>32</v>
       </c>
       <c r="S38" s="4" t="s">
-        <v>81</v>
+        <v>46</v>
       </c>
     </row>
     <row r="39" spans="1:19" x14ac:dyDescent="0.25">
@@ -2587,28 +2564,28 @@
         <v>21</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="F39" s="3" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="G39" s="4" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="H39" s="3" t="s">
         <v>27</v>
       </c>
       <c r="I39" s="4" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="J39" s="4" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="K39" s="5">
         <v>1666667</v>
@@ -2633,7 +2610,7 @@
         <v>32</v>
       </c>
       <c r="S39" s="4" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
     </row>
     <row r="40" spans="1:19" x14ac:dyDescent="0.25">
@@ -2641,31 +2618,31 @@
         <v>34</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="F40" s="3" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="G40" s="4" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="H40" s="3" t="s">
         <v>27</v>
       </c>
       <c r="I40" s="4" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="J40" s="4" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
       <c r="K40" s="5"/>
       <c r="L40" s="5"/>
@@ -2686,7 +2663,7 @@
         <v>32</v>
       </c>
       <c r="S40" s="4" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="41" spans="1:19" x14ac:dyDescent="0.25">
@@ -2697,28 +2674,28 @@
         <v>21</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="E41" s="3" t="s">
         <v>48</v>
       </c>
       <c r="F41" s="3" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="G41" s="4" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="H41" s="3" t="s">
         <v>27</v>
       </c>
       <c r="I41" s="4" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="J41" s="4" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="K41" s="5">
         <v>600068</v>
@@ -2741,7 +2718,7 @@
         <v>32</v>
       </c>
       <c r="S41" s="4" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="42" spans="1:19" x14ac:dyDescent="0.25">
@@ -2752,19 +2729,19 @@
         <v>21</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="F42" s="3" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
       <c r="G42" s="4" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="H42" s="3" t="s">
         <v>27</v>
@@ -2798,7 +2775,7 @@
         <v>32</v>
       </c>
       <c r="S42" s="4" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
     </row>
     <row r="43" spans="1:19" x14ac:dyDescent="0.25">
@@ -2809,19 +2786,19 @@
         <v>21</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="F43" s="3" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="G43" s="4" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="H43" s="3" t="s">
         <v>27</v>
@@ -2830,7 +2807,7 @@
         <v>28</v>
       </c>
       <c r="J43" s="4" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="K43" s="5">
         <v>227273</v>
@@ -2855,7 +2832,7 @@
         <v>32</v>
       </c>
       <c r="S43" s="4" t="s">
-        <v>172</v>
+        <v>72</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add invoice items JSON export with detailed line items and transaction info
</commit_message>
<xml_diff>
--- a/gdt-aggregated-xlsx/hd_purchased_merged.xlsx
+++ b/gdt-aggregated-xlsx/hd_purchased_merged.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="502" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="502" uniqueCount="167">
   <si>
     <t>DANH SÁCH HÓA ĐƠN</t>
   </si>
@@ -115,7 +115,8 @@
     <t>Hóa đơn mới</t>
   </si>
   <si>
-    <t>Hàng hóa, dịch vụ - Xăng E10 RON 95 Mức 3 - 36.265 - Lít - 22.060 - 800.000 - KKKNT</t>
+    <t xml:space="preserve">Họ tên người mua hàng: 51F - 885.92
+Hàng hóa, dịch vụ - Xăng E10 RON 95 Mức 3 - 33.73494 - Lít - 20.750 - 700.000 - KKKNT</t>
   </si>
   <si>
     <t>C26TBA</t>
@@ -145,7 +146,7 @@
     <t>05/06/2026</t>
   </si>
   <si>
-    <t>Hàng hóa, dịch vụ - Dịch vụ phần mềm quản lý và lưu trữ dữ liệu theo học viên (01/06/2026 - 31/05/2027) - 1 - Gói - 1.200.000 - 1.200.000 - KCT</t>
+    <t>Hàng hóa, dịch vụ - Ắc quy GS MF 85D26L - 1 - Cái - 1.666.667 - 1.666.667 - 8%</t>
   </si>
   <si>
     <t>3965</t>
@@ -163,13 +164,15 @@
     <t>26/06/2026</t>
   </si>
   <si>
-    <t xml:space="preserve">Hàng hóa, dịch vụ - Dịch vụ phần mềm quản lý và lưu trữ dữ liệu theo học viên (01/07/2026 - 30/06/2027) - 14 - Gói - 1.200.000 - 16.800.000 - KCT
-Hàng hóa, dịch vụ - Dịch vụ phần mềm quản lý và lưu trữ dữ liệu theo học viên (15/07/2026 - 14/07/2027) - 17 - Gói - 1.200.000 - 20.400.000 - KCT</t>
+    <t>Hàng hóa, dịch vụ - Thu tiền ôn tập trên sân và xe có thiết bị. “Đã giảm 52.200 đồng tương ứng 20% mức tỷ lệ % để tính thuế giá trị gia tăng theo nghị quyết số 204/2025/QH15”. - 9 - Giờ - 580.000</t>
   </si>
   <si>
     <t>4252</t>
   </si>
   <si>
+    <t>Hàng hóa, dịch vụ - Dịch vụ phần mềm quản lý và lưu trữ dữ liệu theo học viên (01/07/2026 - 30/06/2027) - 1 - Gói - 1.200.000 - 1.200.000 - KCT</t>
+  </si>
+  <si>
     <t>C26TBD</t>
   </si>
   <si>
@@ -188,6 +191,10 @@
     <t>53 Nguyễn Đức Thuận, Phường Tân Bình,  TP Hồ Chí Minh, Việt Nam</t>
   </si>
   <si>
+    <t xml:space="preserve">Họ tên người mua hàng: 51K-09402
+Hàng hóa, dịch vụ - Xăng E10 RON95 Mức 3 - 27.896 - Lít - 23.660 - 660.019 - KKKNT</t>
+  </si>
+  <si>
     <t>114100</t>
   </si>
   <si>
@@ -200,8 +207,8 @@
     <t>04/06/2026</t>
   </si>
   <si>
-    <t xml:space="preserve">Hàng hóa, dịch vụ - DO.TTKD037_KD05/M03/2600660900 - Bảo hiểm bắt buộc TNDS của chủ xe 51C45909 - 1 - đơn vị - 4.800.000 - 4.800.000 - 10%
-Hàng hóa, dịch vụ - DO.TTKD037_KD05/M03/2600660900 - Bảo hiểm Tai nạn lái xe và người ngồi trên xe - 1 - đơn vị - 20.000 - 20.000 - KCT</t>
+    <t xml:space="preserve">Họ tên người mua hàng: 51L 32108
+Hàng hóa, dịch vụ - Xăng E10 RON95 Mức 3 - 18.002 - Lít - 23.330 - 420.000 - KKKNT</t>
   </si>
   <si>
     <t>120251</t>
@@ -211,6 +218,23 @@
   </si>
   <si>
     <t>07/06/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Họ tên người mua hàng: 51L 32108
+Hàng hóa, dịch vụ - Xăng E10 RON95 Mức 3 - 15.673 - Lít - 22.330 - 350.000 - KKKNT</t>
+  </si>
+  <si>
+    <t>123723</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Họ tên người mua hàng: 51K 09402
+Hàng hóa, dịch vụ - Xăng E10 RON95 Mức 3 - 35.244 - Lít - 22.330 - 787.000 - KKKNT</t>
+  </si>
+  <si>
+    <t>127104</t>
+  </si>
+  <si>
+    <t>09/06/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Ghi chú, diễn giải - Sửa chữa xe BKS 51A91775 - 0 - 0%
@@ -220,31 +244,20 @@
 Hàng hóa, dịch vụ - Lọc dầu động cơ - 1 - Cái - 187.200 - 187.200 - 8%</t>
   </si>
   <si>
-    <t>123723</t>
-  </si>
-  <si>
-    <t>Hàng hóa, dịch vụ - Xăng E10 RON95 Mức 3 - 35.244 - Lít - 22.330 - 787.000 - KKKNT</t>
-  </si>
-  <si>
-    <t>127104</t>
-  </si>
-  <si>
-    <t>09/06/2026</t>
-  </si>
-  <si>
     <t>134471</t>
   </si>
   <si>
     <t>14/06/2026</t>
   </si>
   <si>
-    <t>Hàng hóa, dịch vụ - Kiểm định Ô tô từ 9 chỗ trở xuống: 51K-126.36 - 1 - Lượt - 227.273 - 227.273 - 8%</t>
+    <t>Hàng hóa, dịch vụ - LỐP ÔTÔ KENDA 205/65R16 95 H KR217 TL - 2 - Cái - 133.333.333 - 2.666.667 - 8%</t>
   </si>
   <si>
     <t>134472</t>
   </si>
   <si>
-    <t>Hàng hóa, dịch vụ - Xăng E10 RON95 Mức 3 - 22.665 - Lít - 22.060 - 500.000 - KKKNT</t>
+    <t xml:space="preserve">Họ tên người mua hàng: 51K-09402
+Hàng hóa, dịch vụ - Xăng E10 RON95 Mức 3 - 22.665 - Lít - 22.060 - 500.000 - KKKNT</t>
   </si>
   <si>
     <t>136322</t>
@@ -256,28 +269,24 @@
     <t>139907</t>
   </si>
   <si>
+    <t xml:space="preserve">Họ tên người mua hàng: 51K 09402
+Hàng hóa, dịch vụ - Xăng E10 RON95 Mức 3 - 31.731 - Lít - 22.060 - 700.000 - KKKNT</t>
+  </si>
+  <si>
     <t>145668</t>
   </si>
   <si>
     <t>21/06/2026</t>
   </si>
   <si>
-    <t xml:space="preserve">Ghi chú, diễn giải - Sửa chữa xe BKS 51H77732 - 0 - 0%
-Hàng hóa, dịch vụ - Bảo dưỡng cấp trung bình ( chỉ vệ sinh thắng đĩa) - 1 - Lượt - 380.000 - 380.000 - 8%
-Hàng hóa, dịch vụ - Dung dịch tẩy rửa bố thắng - 1 - Chai - 90.900 - 90.900 - 8%
-Hàng hóa, dịch vụ - Dầu máy SP 10W-30 (phuy 208L) - 3.3 - Lít - 104.400 - 344.520 - 8%
-Hàng hóa, dịch vụ - Lọc dầu động cơ - 1 - Cái - 187.200 - 187.200 - 8%
-Hàng hóa, dịch vụ - Gioăng làm kín ốc xả dầu - 1 - Cái - 10.800 - 10.800 - 8%
-Hàng hóa, dịch vụ - Lõi lọc gió động cơ - 1 - Cái - 369.900 - 369.900 - 8%</t>
-  </si>
-  <si>
     <t>147715</t>
   </si>
   <si>
     <t>23/06/2026</t>
   </si>
   <si>
-    <t>Hàng hóa, dịch vụ - Xăng E10 RON95 Mức 3 - 26.409 - Lít - 20.750 - 548.000 - KKKNT</t>
+    <t xml:space="preserve">Họ tên người mua hàng: 51L-32108
+Hàng hóa, dịch vụ - Xăng E10 RON95 Mức 3 - 19.277 - Lít - 20.750 - 400.000 - KKKNT</t>
   </si>
   <si>
     <t>149230</t>
@@ -286,16 +295,14 @@
     <t>24/06/2026</t>
   </si>
   <si>
-    <t>Hàng hóa, dịch vụ - Xăng E10 RON95 Mức 3 - 19.277 - Lít - 20.750 - 400.000 - KKKNT</t>
-  </si>
-  <si>
     <t>159219</t>
   </si>
   <si>
     <t>30/06/2026</t>
   </si>
   <si>
-    <t>Hàng hóa, dịch vụ - Xăng E10 RON95 Mức 3 - 25.113 - Lít - 19.910 - 500.000 - KKKNT</t>
+    <t xml:space="preserve">Họ tên người mua hàng: 51L 32108
+Hàng hóa, dịch vụ - Xăng E10 RON95 Mức 3 - 28.3 - Lít - 21.200 - 600.000 - KKKNT</t>
   </si>
   <si>
     <t>C26TTC</t>
@@ -368,9 +375,6 @@
   </si>
   <si>
     <t>7948</t>
-  </si>
-  <si>
-    <t>Hàng hóa, dịch vụ - Thu tiền ôn tập trên sân và xe có thiết bị. “Đã giảm 49.300 đồng tương ứng 20% mức tỷ lệ % để tính thuế giá trị gia tăng theo nghị quyết số 204/2025/QH15”. - 8.5 - Giờ - 580.000 - 4.930.000</t>
   </si>
   <si>
     <t>C26TSH</t>
@@ -479,9 +483,6 @@
     <t>53 Nguyễn Đức Thuận, Phường Tân Bình, Thành phố  Hồ Chí Minh, Việt Nam</t>
   </si>
   <si>
-    <t>Hàng hóa, dịch vụ - Ắc quy GS MF 85D26L - 1 - Cái - 1.666.667 - 1.666.667 - 8%</t>
-  </si>
-  <si>
     <t>C26THL</t>
   </si>
   <si>
@@ -495,6 +496,9 @@
   </si>
   <si>
     <t>53 Nguyễn Đức Thuận, Phường Tân Bình, TP Hồ Chí Minh, Việt Nam.</t>
+  </si>
+  <si>
+    <t>Hàng hóa, dịch vụ - Mực túi MP3554, 1000g - Biasdo - 1 - Túi - 500.000 - 500.000</t>
   </si>
   <si>
     <t>C26TVT</t>
@@ -1087,7 +1091,7 @@
         <v>32</v>
       </c>
       <c r="S12" s="4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="13" spans="1:19" x14ac:dyDescent="0.25">
@@ -1098,19 +1102,19 @@
         <v>21</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="H13" s="3" t="s">
         <v>27</v>
@@ -1119,7 +1123,7 @@
         <v>28</v>
       </c>
       <c r="J13" s="4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="K13" s="5">
         <v>530000</v>
@@ -1144,7 +1148,7 @@
         <v>32</v>
       </c>
       <c r="S13" s="4" t="s">
-        <v>40</v>
+        <v>58</v>
       </c>
     </row>
     <row r="14" spans="1:19" x14ac:dyDescent="0.25">
@@ -1155,19 +1159,19 @@
         <v>21</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="H14" s="3" t="s">
         <v>27</v>
@@ -1176,7 +1180,7 @@
         <v>28</v>
       </c>
       <c r="J14" s="4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="K14" s="5">
         <v>660019</v>
@@ -1201,7 +1205,7 @@
         <v>32</v>
       </c>
       <c r="S14" s="4" t="s">
-        <v>40</v>
+        <v>58</v>
       </c>
     </row>
     <row r="15" spans="1:19" x14ac:dyDescent="0.25">
@@ -1212,19 +1216,19 @@
         <v>21</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="H15" s="3" t="s">
         <v>27</v>
@@ -1233,7 +1237,7 @@
         <v>28</v>
       </c>
       <c r="J15" s="4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="K15" s="5">
         <v>420000</v>
@@ -1258,7 +1262,7 @@
         <v>32</v>
       </c>
       <c r="S15" s="4" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.25">
@@ -1269,19 +1273,19 @@
         <v>21</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="E16" s="3" t="s">
         <v>42</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="H16" s="3" t="s">
         <v>27</v>
@@ -1290,7 +1294,7 @@
         <v>28</v>
       </c>
       <c r="J16" s="4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="K16" s="5">
         <v>700023</v>
@@ -1326,19 +1330,19 @@
         <v>21</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="H17" s="3" t="s">
         <v>27</v>
@@ -1347,7 +1351,7 @@
         <v>28</v>
       </c>
       <c r="J17" s="4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="K17" s="5">
         <v>350000</v>
@@ -1372,7 +1376,7 @@
         <v>32</v>
       </c>
       <c r="S17" s="4" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="18" spans="1:19" x14ac:dyDescent="0.25">
@@ -1383,19 +1387,19 @@
         <v>21</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D18" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="E18" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="E18" s="3" t="s">
-        <v>64</v>
-      </c>
       <c r="F18" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="H18" s="3" t="s">
         <v>27</v>
@@ -1404,7 +1408,7 @@
         <v>28</v>
       </c>
       <c r="J18" s="4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="K18" s="5">
         <v>787000</v>
@@ -1429,7 +1433,7 @@
         <v>32</v>
       </c>
       <c r="S18" s="4" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.25">
@@ -1440,19 +1444,19 @@
         <v>21</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="H19" s="3" t="s">
         <v>27</v>
@@ -1461,7 +1465,7 @@
         <v>28</v>
       </c>
       <c r="J19" s="4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="K19" s="5">
         <v>699956</v>
@@ -1486,7 +1490,7 @@
         <v>32</v>
       </c>
       <c r="S19" s="4" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
     </row>
     <row r="20" spans="1:19" x14ac:dyDescent="0.25">
@@ -1497,19 +1501,19 @@
         <v>21</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="H20" s="3" t="s">
         <v>27</v>
@@ -1518,7 +1522,7 @@
         <v>28</v>
       </c>
       <c r="J20" s="4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="K20" s="5">
         <v>535000</v>
@@ -1543,7 +1547,7 @@
         <v>32</v>
       </c>
       <c r="S20" s="4" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
     </row>
     <row r="21" spans="1:19" x14ac:dyDescent="0.25">
@@ -1554,19 +1558,19 @@
         <v>21</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="H21" s="3" t="s">
         <v>27</v>
@@ -1575,7 +1579,7 @@
         <v>28</v>
       </c>
       <c r="J21" s="4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="K21" s="5">
         <v>500000</v>
@@ -1600,7 +1604,7 @@
         <v>32</v>
       </c>
       <c r="S21" s="4" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="22" spans="1:19" x14ac:dyDescent="0.25">
@@ -1611,19 +1615,19 @@
         <v>21</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G22" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="H22" s="3" t="s">
         <v>27</v>
@@ -1632,7 +1636,7 @@
         <v>28</v>
       </c>
       <c r="J22" s="4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="K22" s="5">
         <v>514373</v>
@@ -1657,7 +1661,7 @@
         <v>32</v>
       </c>
       <c r="S22" s="4" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
     </row>
     <row r="23" spans="1:19" x14ac:dyDescent="0.25">
@@ -1668,19 +1672,19 @@
         <v>21</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="E23" s="3" t="s">
         <v>45</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="H23" s="3" t="s">
         <v>27</v>
@@ -1689,7 +1693,7 @@
         <v>28</v>
       </c>
       <c r="J23" s="4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="K23" s="5">
         <v>700000</v>
@@ -1714,7 +1718,7 @@
         <v>32</v>
       </c>
       <c r="S23" s="4" t="s">
-        <v>46</v>
+        <v>81</v>
       </c>
     </row>
     <row r="24" spans="1:19" x14ac:dyDescent="0.25">
@@ -1725,19 +1729,19 @@
         <v>21</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G24" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="H24" s="3" t="s">
         <v>27</v>
@@ -1746,7 +1750,7 @@
         <v>28</v>
       </c>
       <c r="J24" s="4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="K24" s="5">
         <v>584008</v>
@@ -1771,7 +1775,7 @@
         <v>32</v>
       </c>
       <c r="S24" s="4" t="s">
-        <v>80</v>
+        <v>33</v>
       </c>
     </row>
     <row r="25" spans="1:19" x14ac:dyDescent="0.25">
@@ -1782,19 +1786,19 @@
         <v>21</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G25" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="H25" s="3" t="s">
         <v>27</v>
@@ -1803,7 +1807,7 @@
         <v>28</v>
       </c>
       <c r="J25" s="4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="K25" s="5">
         <v>548000</v>
@@ -1828,7 +1832,7 @@
         <v>32</v>
       </c>
       <c r="S25" s="4" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.25">
@@ -1839,19 +1843,19 @@
         <v>21</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G26" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="H26" s="3" t="s">
         <v>27</v>
@@ -1860,7 +1864,7 @@
         <v>28</v>
       </c>
       <c r="J26" s="4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="K26" s="5">
         <v>400000</v>
@@ -1896,19 +1900,19 @@
         <v>21</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G27" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="H27" s="3" t="s">
         <v>27</v>
@@ -1917,7 +1921,7 @@
         <v>28</v>
       </c>
       <c r="J27" s="4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="K27" s="5">
         <v>500000</v>
@@ -1942,7 +1946,7 @@
         <v>32</v>
       </c>
       <c r="S27" s="4" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="28" spans="1:19" x14ac:dyDescent="0.25">
@@ -1953,25 +1957,25 @@
         <v>21</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="E28" s="3" t="s">
         <v>42</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="G28" s="4" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="H28" s="3" t="s">
         <v>27</v>
       </c>
       <c r="I28" s="4" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="J28" s="4" t="s">
         <v>29</v>
@@ -1999,7 +2003,7 @@
         <v>32</v>
       </c>
       <c r="S28" s="4" t="s">
-        <v>61</v>
+        <v>43</v>
       </c>
     </row>
     <row r="29" spans="1:19" x14ac:dyDescent="0.25">
@@ -2010,25 +2014,25 @@
         <v>21</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D29" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="E29" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="F29" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="G29" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="H29" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="I29" s="4" t="s">
         <v>96</v>
-      </c>
-      <c r="E29" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="F29" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="G29" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="H29" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="I29" s="4" t="s">
-        <v>94</v>
       </c>
       <c r="J29" s="4" t="s">
         <v>29</v>
@@ -2056,7 +2060,7 @@
         <v>32</v>
       </c>
       <c r="S29" s="4" t="s">
-        <v>46</v>
+        <v>81</v>
       </c>
     </row>
     <row r="30" spans="1:19" x14ac:dyDescent="0.25">
@@ -2067,28 +2071,28 @@
         <v>21</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="G30" s="4" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="H30" s="3" t="s">
         <v>27</v>
       </c>
       <c r="I30" s="4" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="J30" s="4" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="K30" s="5">
         <v>1354545</v>
@@ -2111,7 +2115,7 @@
         <v>32</v>
       </c>
       <c r="S30" s="4" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="31" spans="1:19" x14ac:dyDescent="0.25">
@@ -2119,31 +2123,31 @@
         <v>25</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F31" s="3" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="G31" s="4" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="H31" s="3" t="s">
         <v>27</v>
       </c>
       <c r="I31" s="4" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="J31" s="4" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="K31" s="5"/>
       <c r="L31" s="5"/>
@@ -2164,7 +2168,7 @@
         <v>32</v>
       </c>
       <c r="S31" s="4" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="32" spans="1:19" x14ac:dyDescent="0.25">
@@ -2172,31 +2176,31 @@
         <v>26</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D32" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="E32" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="F32" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="G32" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="H32" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="I32" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="J32" s="4" t="s">
         <v>113</v>
-      </c>
-      <c r="E32" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="F32" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="G32" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="H32" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="I32" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="J32" s="4" t="s">
-        <v>111</v>
       </c>
       <c r="K32" s="5"/>
       <c r="L32" s="5"/>
@@ -2217,7 +2221,7 @@
         <v>32</v>
       </c>
       <c r="S32" s="4" t="s">
-        <v>114</v>
+        <v>49</v>
       </c>
     </row>
     <row r="33" spans="1:19" x14ac:dyDescent="0.25">
@@ -2228,19 +2232,19 @@
         <v>21</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="F33" s="3" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G33" s="4" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H33" s="3" t="s">
         <v>27</v>
@@ -2249,7 +2253,7 @@
         <v>28</v>
       </c>
       <c r="J33" s="4" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="K33" s="5">
         <v>138481482</v>
@@ -2274,7 +2278,7 @@
         <v>32</v>
       </c>
       <c r="S33" s="4" t="s">
-        <v>46</v>
+        <v>81</v>
       </c>
     </row>
     <row r="34" spans="1:19" x14ac:dyDescent="0.25">
@@ -2285,25 +2289,25 @@
         <v>21</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="G34" s="4" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="H34" s="3" t="s">
         <v>27</v>
       </c>
       <c r="I34" s="4" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="J34" s="4" t="s">
         <v>29</v>
@@ -2329,7 +2333,7 @@
         <v>32</v>
       </c>
       <c r="S34" s="4" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="35" spans="1:19" x14ac:dyDescent="0.25">
@@ -2340,25 +2344,25 @@
         <v>21</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="G35" s="4" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="H35" s="3" t="s">
         <v>27</v>
       </c>
       <c r="I35" s="4" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="J35" s="4" t="s">
         <v>29</v>
@@ -2384,7 +2388,7 @@
         <v>32</v>
       </c>
       <c r="S35" s="4" t="s">
-        <v>80</v>
+        <v>33</v>
       </c>
     </row>
     <row r="36" spans="1:19" x14ac:dyDescent="0.25">
@@ -2395,19 +2399,19 @@
         <v>21</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="G36" s="4" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="H36" s="3" t="s">
         <v>27</v>
@@ -2416,7 +2420,7 @@
         <v>28</v>
       </c>
       <c r="J36" s="4" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="K36" s="5">
         <v>1383320</v>
@@ -2439,7 +2443,7 @@
         <v>32</v>
       </c>
       <c r="S36" s="4" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="37" spans="1:19" x14ac:dyDescent="0.25">
@@ -2450,25 +2454,25 @@
         <v>21</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="G37" s="4" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H37" s="3" t="s">
         <v>27</v>
       </c>
       <c r="I37" s="4" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="J37" s="4" t="s">
         <v>39</v>
@@ -2496,7 +2500,7 @@
         <v>32</v>
       </c>
       <c r="S37" s="4" t="s">
-        <v>80</v>
+        <v>33</v>
       </c>
     </row>
     <row r="38" spans="1:19" x14ac:dyDescent="0.25">
@@ -2507,19 +2511,19 @@
         <v>21</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="G38" s="4" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="H38" s="3" t="s">
         <v>27</v>
@@ -2553,7 +2557,7 @@
         <v>32</v>
       </c>
       <c r="S38" s="4" t="s">
-        <v>46</v>
+        <v>75</v>
       </c>
     </row>
     <row r="39" spans="1:19" x14ac:dyDescent="0.25">
@@ -2564,28 +2568,28 @@
         <v>21</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F39" s="3" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="G39" s="4" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H39" s="3" t="s">
         <v>27</v>
       </c>
       <c r="I39" s="4" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="J39" s="4" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="K39" s="5">
         <v>1666667</v>
@@ -2610,7 +2614,7 @@
         <v>32</v>
       </c>
       <c r="S39" s="4" t="s">
-        <v>147</v>
+        <v>43</v>
       </c>
     </row>
     <row r="40" spans="1:19" x14ac:dyDescent="0.25">
@@ -2618,7 +2622,7 @@
         <v>34</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C40" s="4" t="s">
         <v>148</v>
@@ -2627,7 +2631,7 @@
         <v>149</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="F40" s="3" t="s">
         <v>150</v>
@@ -2639,7 +2643,7 @@
         <v>27</v>
       </c>
       <c r="I40" s="4" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="J40" s="4" t="s">
         <v>152</v>
@@ -2663,7 +2667,7 @@
         <v>32</v>
       </c>
       <c r="S40" s="4" t="s">
-        <v>61</v>
+        <v>153</v>
       </c>
     </row>
     <row r="41" spans="1:19" x14ac:dyDescent="0.25">
@@ -2674,28 +2678,28 @@
         <v>21</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E41" s="3" t="s">
         <v>48</v>
       </c>
       <c r="F41" s="3" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="G41" s="4" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="H41" s="3" t="s">
         <v>27</v>
       </c>
       <c r="I41" s="4" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="J41" s="4" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="K41" s="5">
         <v>600068</v>
@@ -2718,7 +2722,7 @@
         <v>32</v>
       </c>
       <c r="S41" s="4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="42" spans="1:19" x14ac:dyDescent="0.25">
@@ -2729,19 +2733,19 @@
         <v>21</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F42" s="3" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="G42" s="4" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="H42" s="3" t="s">
         <v>27</v>
@@ -2775,7 +2779,7 @@
         <v>32</v>
       </c>
       <c r="S42" s="4" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
     </row>
     <row r="43" spans="1:19" x14ac:dyDescent="0.25">
@@ -2786,19 +2790,19 @@
         <v>21</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="F43" s="3" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="G43" s="4" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="H43" s="3" t="s">
         <v>27</v>
@@ -2807,7 +2811,7 @@
         <v>28</v>
       </c>
       <c r="J43" s="4" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="K43" s="5">
         <v>227273</v>
@@ -2832,7 +2836,7 @@
         <v>32</v>
       </c>
       <c r="S43" s="4" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add buyer name extraction and mapping functionality for invoices
</commit_message>
<xml_diff>
--- a/gdt-aggregated-xlsx/hd_purchased_merged.xlsx
+++ b/gdt-aggregated-xlsx/hd_purchased_merged.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="502" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="540" uniqueCount="174">
   <si>
     <t>DANH SÁCH HÓA ĐƠN</t>
   </si>
@@ -79,6 +79,9 @@
     <t>Chi tiết hoá đơn</t>
   </si>
   <si>
+    <t>Họ tên người mua hàng</t>
+  </si>
+  <si>
     <t>1</t>
   </si>
   <si>
@@ -115,8 +118,10 @@
     <t>Hóa đơn mới</t>
   </si>
   <si>
-    <t xml:space="preserve">Họ tên người mua hàng: 51F - 885.92
-Hàng hóa, dịch vụ - Xăng E10 RON 95 Mức 3 - 33.73494 - Lít - 20.750 - 700.000 - KKKNT</t>
+    <t>Hàng hóa, dịch vụ - Xăng E10 RON 95 Mức 3 - 33.73494 - Lít - 20.750 - 700.000 - KKKNT</t>
+  </si>
+  <si>
+    <t>51F - 885.92</t>
   </si>
   <si>
     <t>C26TBA</t>
@@ -140,6 +145,9 @@
     <t>Hàng hóa, dịch vụ - Dịch vụ sửa chữa - 1 - Gói - 850.000 - 850.000 - 8%</t>
   </si>
   <si>
+    <t/>
+  </si>
+  <si>
     <t>3662</t>
   </si>
   <si>
@@ -191,8 +199,10 @@
     <t>53 Nguyễn Đức Thuận, Phường Tân Bình,  TP Hồ Chí Minh, Việt Nam</t>
   </si>
   <si>
-    <t xml:space="preserve">Họ tên người mua hàng: 51K-09402
-Hàng hóa, dịch vụ - Xăng E10 RON95 Mức 3 - 27.896 - Lít - 23.660 - 660.019 - KKKNT</t>
+    <t>Hàng hóa, dịch vụ - Xăng E10 RON95 Mức 3 - 27.896 - Lít - 23.660 - 660.019 - KKKNT</t>
+  </si>
+  <si>
+    <t>51K-09402</t>
   </si>
   <si>
     <t>114100</t>
@@ -207,8 +217,10 @@
     <t>04/06/2026</t>
   </si>
   <si>
-    <t xml:space="preserve">Họ tên người mua hàng: 51L 32108
-Hàng hóa, dịch vụ - Xăng E10 RON95 Mức 3 - 18.002 - Lít - 23.330 - 420.000 - KKKNT</t>
+    <t>Hàng hóa, dịch vụ - Xăng E10 RON95 Mức 3 - 18.002 - Lít - 23.330 - 420.000 - KKKNT</t>
+  </si>
+  <si>
+    <t>51L 32108</t>
   </si>
   <si>
     <t>120251</t>
@@ -220,15 +232,16 @@
     <t>07/06/2026</t>
   </si>
   <si>
-    <t xml:space="preserve">Họ tên người mua hàng: 51L 32108
-Hàng hóa, dịch vụ - Xăng E10 RON95 Mức 3 - 15.673 - Lít - 22.330 - 350.000 - KKKNT</t>
+    <t>Hàng hóa, dịch vụ - Xăng E10 RON95 Mức 3 - 15.673 - Lít - 22.330 - 350.000 - KKKNT</t>
   </si>
   <si>
     <t>123723</t>
   </si>
   <si>
-    <t xml:space="preserve">Họ tên người mua hàng: 51K 09402
-Hàng hóa, dịch vụ - Xăng E10 RON95 Mức 3 - 35.244 - Lít - 22.330 - 787.000 - KKKNT</t>
+    <t>Hàng hóa, dịch vụ - Xăng E10 RON95 Mức 3 - 35.244 - Lít - 22.330 - 787.000 - KKKNT</t>
+  </si>
+  <si>
+    <t>51K 09402</t>
   </si>
   <si>
     <t>127104</t>
@@ -237,11 +250,11 @@
     <t>09/06/2026</t>
   </si>
   <si>
-    <t xml:space="preserve">Ghi chú, diễn giải - Sửa chữa xe BKS 51A91775 - 0 - 0%
-Hàng hóa, dịch vụ - Bảo dưỡng cấp trung bình kdd - 1 - Lượt - 250.000 - 250.000 - 8%
-Hàng hóa, dịch vụ - Dầu máy SP 10W-30 (phuy 208L) - 3.7 - Lít - 104.400 - 386.280 - 8%
-Hàng hóa, dịch vụ - Gioăng làm kín ốc xả dầu - 1 - Cái - 10.800 - 10.800 - 8%
-Hàng hóa, dịch vụ - Lọc dầu động cơ - 1 - Cái - 187.200 - 187.200 - 8%</t>
+    <t xml:space="preserve">1. Ghi chú, diễn giải - Sửa chữa xe BKS 51A91775 - 0 - 0%
+2. Hàng hóa, dịch vụ - Bảo dưỡng cấp trung bình kdd - 1 - Lượt - 250.000 - 250.000 - 8%
+3. Hàng hóa, dịch vụ - Dầu máy SP 10W-30 (phuy 208L) - 3.7 - Lít - 104.400 - 386.280 - 8%
+4. Hàng hóa, dịch vụ - Gioăng làm kín ốc xả dầu - 1 - Cái - 10.800 - 10.800 - 8%
+5. Hàng hóa, dịch vụ - Lọc dầu động cơ - 1 - Cái - 187.200 - 187.200 - 8%</t>
   </si>
   <si>
     <t>134471</t>
@@ -256,8 +269,7 @@
     <t>134472</t>
   </si>
   <si>
-    <t xml:space="preserve">Họ tên người mua hàng: 51K-09402
-Hàng hóa, dịch vụ - Xăng E10 RON95 Mức 3 - 22.665 - Lít - 22.060 - 500.000 - KKKNT</t>
+    <t>Hàng hóa, dịch vụ - Xăng E10 RON95 Mức 3 - 22.665 - Lít - 22.060 - 500.000 - KKKNT</t>
   </si>
   <si>
     <t>136322</t>
@@ -269,8 +281,7 @@
     <t>139907</t>
   </si>
   <si>
-    <t xml:space="preserve">Họ tên người mua hàng: 51K 09402
-Hàng hóa, dịch vụ - Xăng E10 RON95 Mức 3 - 31.731 - Lít - 22.060 - 700.000 - KKKNT</t>
+    <t>Hàng hóa, dịch vụ - Xăng E10 RON95 Mức 3 - 31.731 - Lít - 22.060 - 700.000 - KKKNT</t>
   </si>
   <si>
     <t>145668</t>
@@ -285,8 +296,10 @@
     <t>23/06/2026</t>
   </si>
   <si>
-    <t xml:space="preserve">Họ tên người mua hàng: 51L-32108
-Hàng hóa, dịch vụ - Xăng E10 RON95 Mức 3 - 19.277 - Lít - 20.750 - 400.000 - KKKNT</t>
+    <t>Hàng hóa, dịch vụ - Xăng E10 RON95 Mức 3 - 19.277 - Lít - 20.750 - 400.000 - KKKNT</t>
+  </si>
+  <si>
+    <t>51L-32108</t>
   </si>
   <si>
     <t>149230</t>
@@ -301,8 +314,7 @@
     <t>30/06/2026</t>
   </si>
   <si>
-    <t xml:space="preserve">Họ tên người mua hàng: 51L 32108
-Hàng hóa, dịch vụ - Xăng E10 RON95 Mức 3 - 28.3 - Lít - 21.200 - 600.000 - KKKNT</t>
+    <t>Hàng hóa, dịch vụ - Xăng E10 RON95 Mức 3 - 28.3 - Lít - 21.200 - 600.000 - KKKNT</t>
   </si>
   <si>
     <t>C26TTC</t>
@@ -410,11 +422,11 @@
     <t>Trung Tâm Giáo Dục Nghề Nghiệp Bách Việt</t>
   </si>
   <si>
-    <t xml:space="preserve">Ghi chú, diễn giải - Sửa chữa xe BKS 51A91775 - 0 - 0%
-Hàng hóa, dịch vụ - Bảo dưỡng cấp trung bình  kdd - 1 - Lượt - 250.000 - 250.000 - 8%
-Hàng hóa, dịch vụ - Dầu máy SP 10W-30 (phuy 208L) - 3.7 - Lít - 104.400 - 386.280 - 8%
-Hàng hóa, dịch vụ - Gioăng làm kín ốc xả dầu - 1 - Cái - 10.800 - 10.800 - 8%
-Hàng hóa, dịch vụ - Lọc dầu động cơ - 1 - Cái - 187.200 - 187.200 - 8%</t>
+    <t xml:space="preserve">1. Ghi chú, diễn giải - Sửa chữa xe BKS 51A91775 - 0 - 0%
+2. Hàng hóa, dịch vụ - Bảo dưỡng cấp trung bình  kdd - 1 - Lượt - 250.000 - 250.000 - 8%
+3. Hàng hóa, dịch vụ - Dầu máy SP 10W-30 (phuy 208L) - 3.7 - Lít - 104.400 - 386.280 - 8%
+4. Hàng hóa, dịch vụ - Gioăng làm kín ốc xả dầu - 1 - Cái - 10.800 - 10.800 - 8%
+5. Hàng hóa, dịch vụ - Lọc dầu động cơ - 1 - Cái - 187.200 - 187.200 - 8%</t>
   </si>
   <si>
     <t>9203</t>
@@ -429,13 +441,13 @@
     <t>53 Nguyễn Đức Thuận, Phường Tân Bình, Thành Phố  Hồ Chí Minh, Việt Nam</t>
   </si>
   <si>
-    <t xml:space="preserve">Ghi chú, diễn giải - Sửa chữa xe BKS 51H77732 - 0 - 0%
-Hàng hóa, dịch vụ - Bảo dưỡng cấp trung bình  ( chỉ vệ sinh thắng đĩa) - 1 - Lượt - 380.000 - 380.000 - 8%
-Hàng hóa, dịch vụ - Dung dịch tẩy rửa bố thắng - 1 - Chai - 90.900 - 90.900 - 8%
-Hàng hóa, dịch vụ - Dầu máy SP 10W-30 (phuy 208L) - 3.3 - Lít - 104.400 - 344.520 - 8%
-Hàng hóa, dịch vụ - Lọc dầu động cơ - 1 - Cái - 187.200 - 187.200 - 8%
-Hàng hóa, dịch vụ - Gioăng làm kín ốc xả dầu - 1 - Cái - 10.800 - 10.800 - 8%
-Hàng hóa, dịch vụ - Lõi lọc gió động cơ - 1 - Cái - 369.900 - 369.900 - 8%</t>
+    <t xml:space="preserve">1. Ghi chú, diễn giải - Sửa chữa xe BKS 51H77732 - 0 - 0%
+2. Hàng hóa, dịch vụ - Bảo dưỡng cấp trung bình  ( chỉ vệ sinh thắng đĩa) - 1 - Lượt - 380.000 - 380.000 - 8%
+3. Hàng hóa, dịch vụ - Dung dịch tẩy rửa bố thắng - 1 - Chai - 90.900 - 90.900 - 8%
+4. Hàng hóa, dịch vụ - Dầu máy SP 10W-30 (phuy 208L) - 3.3 - Lít - 104.400 - 344.520 - 8%
+5. Hàng hóa, dịch vụ - Lọc dầu động cơ - 1 - Cái - 187.200 - 187.200 - 8%
+6. Hàng hóa, dịch vụ - Gioăng làm kín ốc xả dầu - 1 - Cái - 10.800 - 10.800 - 8%
+7. Hàng hóa, dịch vụ - Lõi lọc gió động cơ - 1 - Cái - 369.900 - 369.900 - 8%</t>
   </si>
   <si>
     <t>C26TYY</t>
@@ -597,7 +609,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -613,6 +625,9 @@
     </xf>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -633,7 +648,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A3:S43"/>
+  <dimension ref="A1:T43"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
   <cols>
     <col min="1" max="1" width="7.8125" customWidth="1"/>
@@ -647,7 +662,9 @@
     <col min="19" max="19" width="50.78125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="1" spans="20:20" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="20:20" x14ac:dyDescent="0.25"/>
+    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -670,7 +687,7 @@
       <c r="R3"/>
       <c r="S3"/>
     </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>1</v>
       </c>
@@ -693,7 +710,8 @@
       <c r="R4"/>
       <c r="S4"/>
     </row>
-    <row r="6" ht="50" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="5" spans="20:20" x14ac:dyDescent="0.25"/>
+    <row r="6" ht="50" customHeight="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>2</v>
       </c>
@@ -751,37 +769,40 @@
       <c r="S6" s="2" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="T6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
         <v>1</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J7" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="K7" s="5">
         <v>800000</v>
@@ -797,48 +818,51 @@
         <v>800000</v>
       </c>
       <c r="P7" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="Q7" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="R7" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="S7" s="4" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+      <c r="T7" s="6" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
         <v>2</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I8" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J8" s="4" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="K8" s="5">
         <v>850000</v>
@@ -854,48 +878,51 @@
         <v>918000</v>
       </c>
       <c r="P8" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="Q8" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="R8" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="S8" s="4" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
+        <v>42</v>
+      </c>
+      <c r="T8" s="6" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A9" s="3">
         <v>3</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D9" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="I9" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="J9" s="4" t="s">
         <v>41</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="G9" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="H9" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="I9" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="J9" s="4" t="s">
-        <v>39</v>
       </c>
       <c r="K9" s="5">
         <v>1200000</v>
@@ -911,48 +938,51 @@
         <v>1200000</v>
       </c>
       <c r="P9" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="Q9" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="R9" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="S9" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="T9" s="6" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A10" s="3">
         <v>4</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J10" s="4" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="K10" s="5">
         <v>3600000</v>
@@ -968,48 +998,51 @@
         <v>3600000</v>
       </c>
       <c r="P10" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="Q10" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="R10" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="S10" s="4" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.25">
+        <v>49</v>
+      </c>
+      <c r="T10" s="6" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A11" s="3">
         <v>5</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I11" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J11" s="4" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="K11" s="5">
         <v>37200000</v>
@@ -1025,48 +1058,51 @@
         <v>37200000</v>
       </c>
       <c r="P11" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="Q11" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="R11" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="S11" s="4" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.25">
+        <v>52</v>
+      </c>
+      <c r="T11" s="6" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A12" s="3">
         <v>6</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I12" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J12" s="4" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="K12" s="5">
         <v>1200000</v>
@@ -1082,48 +1118,51 @@
         <v>1200000</v>
       </c>
       <c r="P12" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="Q12" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="R12" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="S12" s="4" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="13" spans="1:19" x14ac:dyDescent="0.25">
+        <v>54</v>
+      </c>
+      <c r="T12" s="6" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A13" s="3">
         <v>7</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I13" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J13" s="4" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="K13" s="5">
         <v>530000</v>
@@ -1139,48 +1178,51 @@
         <v>530000</v>
       </c>
       <c r="P13" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="Q13" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="R13" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="S13" s="4" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.25">
+        <v>61</v>
+      </c>
+      <c r="T13" s="6" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A14" s="3">
         <v>8</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="D14" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="G14" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="E14" s="3" t="s">
+      <c r="H14" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="I14" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="J14" s="4" t="s">
         <v>60</v>
-      </c>
-      <c r="F14" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="G14" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="H14" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="I14" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="J14" s="4" t="s">
-        <v>57</v>
       </c>
       <c r="K14" s="5">
         <v>660019</v>
@@ -1196,48 +1238,51 @@
         <v>660019</v>
       </c>
       <c r="P14" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="Q14" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="R14" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="S14" s="4" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.25">
+        <v>61</v>
+      </c>
+      <c r="T14" s="6" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A15" s="3">
         <v>9</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I15" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J15" s="4" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="K15" s="5">
         <v>420000</v>
@@ -1253,48 +1298,51 @@
         <v>420000</v>
       </c>
       <c r="P15" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="Q15" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="R15" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="S15" s="4" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="16" spans="1:19" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+      <c r="T15" s="6" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A16" s="3">
         <v>10</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I16" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J16" s="4" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="K16" s="5">
         <v>700023</v>
@@ -1310,48 +1358,51 @@
         <v>700023</v>
       </c>
       <c r="P16" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="Q16" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="R16" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="S16" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="T16" s="6" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="17" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A17" s="3">
         <v>11</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I17" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J17" s="4" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="K17" s="5">
         <v>350000</v>
@@ -1367,48 +1418,51 @@
         <v>350000</v>
       </c>
       <c r="P17" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="Q17" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="R17" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="S17" s="4" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="18" spans="1:19" x14ac:dyDescent="0.25">
+        <v>72</v>
+      </c>
+      <c r="T17" s="6" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="18" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A18" s="3">
         <v>12</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I18" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J18" s="4" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="K18" s="5">
         <v>787000</v>
@@ -1424,48 +1478,51 @@
         <v>787000</v>
       </c>
       <c r="P18" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="Q18" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="R18" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="S18" s="4" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="19" spans="1:19" x14ac:dyDescent="0.25">
+        <v>74</v>
+      </c>
+      <c r="T18" s="6" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="19" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A19" s="3">
         <v>13</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I19" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J19" s="4" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="K19" s="5">
         <v>699956</v>
@@ -1481,48 +1538,51 @@
         <v>699956</v>
       </c>
       <c r="P19" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="Q19" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="R19" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="S19" s="4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="20" spans="1:19" x14ac:dyDescent="0.25">
+        <v>78</v>
+      </c>
+      <c r="T19" s="6" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="20" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A20" s="3">
         <v>14</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I20" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J20" s="4" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="K20" s="5">
         <v>535000</v>
@@ -1538,48 +1598,51 @@
         <v>535000</v>
       </c>
       <c r="P20" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="Q20" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="R20" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="S20" s="4" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="21" spans="1:19" x14ac:dyDescent="0.25">
+        <v>81</v>
+      </c>
+      <c r="T20" s="6" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="21" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A21" s="3">
         <v>15</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I21" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J21" s="4" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="K21" s="5">
         <v>500000</v>
@@ -1595,48 +1658,51 @@
         <v>500000</v>
       </c>
       <c r="P21" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="Q21" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="R21" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="S21" s="4" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="22" spans="1:19" x14ac:dyDescent="0.25">
+        <v>83</v>
+      </c>
+      <c r="T21" s="6" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="22" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A22" s="3">
         <v>16</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="G22" s="4" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="H22" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I22" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J22" s="4" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="K22" s="5">
         <v>514373</v>
@@ -1652,48 +1718,51 @@
         <v>514373</v>
       </c>
       <c r="P22" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="Q22" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="R22" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="S22" s="4" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="23" spans="1:19" x14ac:dyDescent="0.25">
+        <v>81</v>
+      </c>
+      <c r="T22" s="6" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="23" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A23" s="3">
         <v>17</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I23" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J23" s="4" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="K23" s="5">
         <v>700000</v>
@@ -1709,48 +1778,51 @@
         <v>700000</v>
       </c>
       <c r="P23" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="Q23" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="R23" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="S23" s="4" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="24" spans="1:19" x14ac:dyDescent="0.25">
+        <v>87</v>
+      </c>
+      <c r="T23" s="6" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="24" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A24" s="3">
         <v>18</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="G24" s="4" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="H24" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I24" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J24" s="4" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="K24" s="5">
         <v>584008</v>
@@ -1766,48 +1838,51 @@
         <v>584008</v>
       </c>
       <c r="P24" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="Q24" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="R24" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="S24" s="4" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="25" spans="1:19" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+      <c r="T24" s="6" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="25" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A25" s="3">
         <v>19</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="G25" s="4" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I25" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J25" s="4" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="K25" s="5">
         <v>548000</v>
@@ -1823,48 +1898,51 @@
         <v>548000</v>
       </c>
       <c r="P25" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="Q25" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="R25" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="S25" s="4" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="26" spans="1:19" x14ac:dyDescent="0.25">
+        <v>92</v>
+      </c>
+      <c r="T25" s="6" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="26" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A26" s="3">
         <v>20</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="G26" s="4" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="H26" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I26" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J26" s="4" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="K26" s="5">
         <v>400000</v>
@@ -1880,48 +1958,51 @@
         <v>400000</v>
       </c>
       <c r="P26" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="Q26" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="R26" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="S26" s="4" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="27" spans="1:19" x14ac:dyDescent="0.25">
+        <v>92</v>
+      </c>
+      <c r="T26" s="6" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="27" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A27" s="3">
         <v>21</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="G27" s="4" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="H27" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I27" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J27" s="4" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="K27" s="5">
         <v>500000</v>
@@ -1937,48 +2018,51 @@
         <v>500000</v>
       </c>
       <c r="P27" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q27" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="R27" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="S27" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="T27" s="6" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="28" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A28" s="3">
+        <v>22</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="E28" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="F28" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="G28" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="H28" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="I28" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="J28" s="4" t="s">
         <v>30</v>
-      </c>
-      <c r="Q27" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="R27" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="S27" s="4" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="28" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A28" s="3">
-        <v>22</v>
-      </c>
-      <c r="B28" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C28" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="D28" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="E28" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="F28" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="G28" s="4" t="s">
-        <v>95</v>
-      </c>
-      <c r="H28" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="I28" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="J28" s="4" t="s">
-        <v>29</v>
       </c>
       <c r="K28" s="5">
         <v>4820000</v>
@@ -1994,48 +2078,51 @@
         <v>5300000</v>
       </c>
       <c r="P28" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="Q28" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="R28" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="S28" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="T28" s="6" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="29" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A29" s="3">
         <v>23</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>100</v>
+        <v>107</v>
       </c>
       <c r="G29" s="4" t="s">
-        <v>101</v>
+        <v>108</v>
       </c>
       <c r="H29" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I29" s="4" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="J29" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="K29" s="5">
         <v>952800</v>
@@ -2051,48 +2138,51 @@
         <v>1048080</v>
       </c>
       <c r="P29" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="Q29" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="R29" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="S29" s="4" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="30" spans="1:19" x14ac:dyDescent="0.25">
+        <v>87</v>
+      </c>
+      <c r="T29" s="6" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="30" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A30" s="3">
         <v>24</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>102</v>
+        <v>109</v>
       </c>
       <c r="D30" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="E30" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="F30" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="G30" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="H30" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="I30" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="E30" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="F30" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="G30" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="H30" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="I30" s="4" t="s">
-        <v>96</v>
-      </c>
       <c r="J30" s="4" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="K30" s="5">
         <v>1354545</v>
@@ -2106,48 +2196,51 @@
         <v>1490000</v>
       </c>
       <c r="P30" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="Q30" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="R30" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="S30" s="4" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="31" spans="1:19" x14ac:dyDescent="0.25">
+        <v>83</v>
+      </c>
+      <c r="T30" s="6" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="31" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A31" s="3">
         <v>25</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="F31" s="3" t="s">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="G31" s="4" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
       <c r="H31" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I31" s="4" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="J31" s="4" t="s">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="K31" s="5"/>
       <c r="L31" s="5"/>
@@ -2159,48 +2252,51 @@
         <v>5167800</v>
       </c>
       <c r="P31" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="Q31" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="R31" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="S31" s="4" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="32" spans="1:19" x14ac:dyDescent="0.25">
+        <v>121</v>
+      </c>
+      <c r="T31" s="6" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="32" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A32" s="3">
         <v>26</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="F32" s="3" t="s">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="G32" s="4" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
       <c r="H32" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I32" s="4" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="J32" s="4" t="s">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="K32" s="5"/>
       <c r="L32" s="5"/>
@@ -2212,48 +2308,51 @@
         <v>4880700</v>
       </c>
       <c r="P32" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="Q32" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="R32" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="S32" s="4" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="33" spans="1:19" x14ac:dyDescent="0.25">
+        <v>52</v>
+      </c>
+      <c r="T32" s="6" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="33" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A33" s="3">
         <v>27</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="F33" s="3" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
       <c r="G33" s="4" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="H33" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I33" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J33" s="4" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="K33" s="5">
         <v>138481482</v>
@@ -2269,48 +2368,51 @@
         <v>149560000</v>
       </c>
       <c r="P33" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q33" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="R33" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="S33" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="T33" s="6" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="34" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A34" s="3">
+        <v>28</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="E34" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="F34" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="G34" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="H34" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="I34" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="J34" s="4" t="s">
         <v>30</v>
-      </c>
-      <c r="Q33" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="R33" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="S33" s="4" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="34" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A34" s="3">
-        <v>28</v>
-      </c>
-      <c r="B34" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C34" s="4" t="s">
-        <v>121</v>
-      </c>
-      <c r="D34" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="E34" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="F34" s="3" t="s">
-        <v>124</v>
-      </c>
-      <c r="G34" s="4" t="s">
-        <v>125</v>
-      </c>
-      <c r="H34" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="I34" s="4" t="s">
-        <v>126</v>
-      </c>
-      <c r="J34" s="4" t="s">
-        <v>29</v>
       </c>
       <c r="K34" s="5">
         <v>834280</v>
@@ -2324,48 +2426,51 @@
         <v>901022</v>
       </c>
       <c r="P34" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="Q34" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="R34" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="S34" s="4" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="35" spans="1:19" x14ac:dyDescent="0.25">
+        <v>134</v>
+      </c>
+      <c r="T34" s="6" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="35" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A35" s="3">
         <v>29</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>121</v>
+        <v>128</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="E35" s="3" t="s">
-        <v>129</v>
+        <v>136</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>124</v>
+        <v>131</v>
       </c>
       <c r="G35" s="4" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="H35" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I35" s="4" t="s">
-        <v>126</v>
+        <v>133</v>
       </c>
       <c r="J35" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="K35" s="5">
         <v>754120</v>
@@ -2379,48 +2484,51 @@
         <v>814450</v>
       </c>
       <c r="P35" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="Q35" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="R35" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="S35" s="4" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="36" spans="1:19" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+      <c r="T35" s="6" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="36" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A36" s="3">
         <v>30</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>121</v>
+        <v>128</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>124</v>
+        <v>131</v>
       </c>
       <c r="G36" s="4" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="H36" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I36" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J36" s="4" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="K36" s="5">
         <v>1383320</v>
@@ -2434,48 +2542,51 @@
         <v>1493986</v>
       </c>
       <c r="P36" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="Q36" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="R36" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="S36" s="4" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="37" spans="1:19" x14ac:dyDescent="0.25">
+        <v>139</v>
+      </c>
+      <c r="T36" s="6" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="37" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A37" s="3">
         <v>31</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>135</v>
+        <v>142</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="G37" s="4" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="H37" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I37" s="4" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="J37" s="4" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="K37" s="5">
         <v>700000</v>
@@ -2491,48 +2602,51 @@
         <v>700000</v>
       </c>
       <c r="P37" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="Q37" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="R37" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="S37" s="4" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="38" spans="1:19" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+      <c r="T37" s="6" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="38" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A38" s="3">
         <v>32</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>138</v>
+        <v>145</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>139</v>
+        <v>146</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="G38" s="4" t="s">
-        <v>141</v>
+        <v>148</v>
       </c>
       <c r="H38" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I38" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J38" s="4" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="K38" s="5">
         <v>2666667</v>
@@ -2548,48 +2662,51 @@
         <v>2880000</v>
       </c>
       <c r="P38" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="Q38" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="R38" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="S38" s="4" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="39" spans="1:19" x14ac:dyDescent="0.25">
+        <v>81</v>
+      </c>
+      <c r="T38" s="6" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="39" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A39" s="3">
         <v>33</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>143</v>
+        <v>150</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>144</v>
+        <v>151</v>
       </c>
       <c r="F39" s="3" t="s">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="G39" s="4" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="H39" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I39" s="4" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="J39" s="4" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="K39" s="5">
         <v>1666667</v>
@@ -2605,48 +2722,51 @@
         <v>1800000</v>
       </c>
       <c r="P39" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="Q39" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="R39" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="S39" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="T39" s="6" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="40" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A40" s="3">
         <v>34</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="F40" s="3" t="s">
-        <v>150</v>
+        <v>157</v>
       </c>
       <c r="G40" s="4" t="s">
-        <v>151</v>
+        <v>158</v>
       </c>
       <c r="H40" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I40" s="4" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="J40" s="4" t="s">
-        <v>152</v>
+        <v>159</v>
       </c>
       <c r="K40" s="5"/>
       <c r="L40" s="5"/>
@@ -2658,48 +2778,51 @@
         <v>500000</v>
       </c>
       <c r="P40" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="Q40" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="R40" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="S40" s="4" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="41" spans="1:19" x14ac:dyDescent="0.25">
+        <v>160</v>
+      </c>
+      <c r="T40" s="6" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="41" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A41" s="3">
         <v>35</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>154</v>
+        <v>161</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>155</v>
+        <v>162</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="F41" s="3" t="s">
-        <v>156</v>
+        <v>163</v>
       </c>
       <c r="G41" s="4" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
       <c r="H41" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I41" s="4" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="J41" s="4" t="s">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="K41" s="5">
         <v>600068</v>
@@ -2713,48 +2836,51 @@
         <v>600068</v>
       </c>
       <c r="P41" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="Q41" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="R41" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="S41" s="4" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="42" spans="1:19" x14ac:dyDescent="0.25">
+        <v>54</v>
+      </c>
+      <c r="T41" s="6" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="42" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A42" s="3">
         <v>36</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>158</v>
+        <v>165</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="F42" s="3" t="s">
-        <v>160</v>
+        <v>167</v>
       </c>
       <c r="G42" s="4" t="s">
-        <v>161</v>
+        <v>168</v>
       </c>
       <c r="H42" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I42" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J42" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="K42" s="5">
         <v>227273</v>
@@ -2770,48 +2896,51 @@
         <v>285455</v>
       </c>
       <c r="P42" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="Q42" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="R42" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="S42" s="4" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="43" spans="1:19" x14ac:dyDescent="0.25">
+        <v>78</v>
+      </c>
+      <c r="T42" s="6" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="43" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A43" s="3">
         <v>37</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>162</v>
+        <v>169</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>163</v>
+        <v>170</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="F43" s="3" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="G43" s="4" t="s">
-        <v>165</v>
+        <v>172</v>
       </c>
       <c r="H43" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I43" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J43" s="4" t="s">
-        <v>166</v>
+        <v>173</v>
       </c>
       <c r="K43" s="5">
         <v>227273</v>
@@ -2827,16 +2956,19 @@
         <v>285455</v>
       </c>
       <c r="P43" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="Q43" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="R43" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="S43" s="4" t="s">
-        <v>75</v>
+        <v>81</v>
+      </c>
+      <c r="T43" s="6" t="s">
+        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>